<commit_message>
Refactor backend into flat modules; refresh dataset, docs and Claude tooling
- Flatten backend/app into one module per concern (loaders, ingest, search,
  answer, guardrails, feedback, metrics, evals, api, db, llm, rules, schemas)
- Dataset quality pass: 24 meetings + 16 OOXML docs, re-dated to 2026
  (user-approved); golden eval set updated to match
- Docs: TECH.md, CODE_REVIEW.md, rewritten MEASUREMENT.md, stale paths and
  dates fixed in TASKS.md / backend README, refreshed project-status memory
- Claude Code: ruff PostToolUse hook and /verify project skill

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/documents/xlsx/action_item_tracker.xlsx
+++ b/data/documents/xlsx/action_item_tracker.xlsx
@@ -1,14 +1,419 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <workbookPr/>
   <sheets>
-    <sheet name="action_item_tracker" sheetId="1" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="action_item_tracker" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
+  <definedNames/>
 </workbook>
+</file>
+
+<file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <numFmts count="0"/>
+  <fonts count="1">
+    <font>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <color theme="1"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+  </fonts>
+  <fills count="2">
+    <fill>
+      <patternFill/>
+    </fill>
+    <fill>
+      <patternFill patternType="gray125"/>
+    </fill>
+  </fills>
+  <borders count="1">
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+  </borders>
+  <cellStyleXfs count="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+  </cellStyleXfs>
+  <cellXfs count="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+  </cellXfs>
+  <cellStyles count="1">
+    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
+  </cellStyles>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
+  <colors>
+    <indexedColors>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008000"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00808000"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="00C0C0C0"/>
+      <rgbColor rgb="00808080"/>
+      <rgbColor rgb="009999FF"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00FFFFCC"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00660066"/>
+      <rgbColor rgb="00FF8080"/>
+      <rgbColor rgb="000066CC"/>
+      <rgbColor rgb="00CCCCFF"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="0000CCFF"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00CCFFCC"/>
+      <rgbColor rgb="00FFFF99"/>
+      <rgbColor rgb="0099CCFF"/>
+      <rgbColor rgb="00FF99CC"/>
+      <rgbColor rgb="00CC99FF"/>
+      <rgbColor rgb="00FFCC99"/>
+      <rgbColor rgb="003366FF"/>
+      <rgbColor rgb="0033CCCC"/>
+      <rgbColor rgb="0099CC00"/>
+      <rgbColor rgb="00FFCC00"/>
+      <rgbColor rgb="00FF9900"/>
+      <rgbColor rgb="00FF6600"/>
+      <rgbColor rgb="00666699"/>
+      <rgbColor rgb="00969696"/>
+      <rgbColor rgb="00003366"/>
+      <rgbColor rgb="00339966"/>
+      <rgbColor rgb="00003300"/>
+      <rgbColor rgb="00333300"/>
+      <rgbColor rgb="00993300"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00333399"/>
+      <rgbColor rgb="00333333"/>
+    </indexedColors>
+  </colors>
+</styleSheet>
+</file>
+
+<file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+  <a:themeElements>
+    <a:clrScheme name="Office">
+      <a:dk1>
+        <a:sysClr val="windowText" lastClr="000000"/>
+      </a:dk1>
+      <a:lt1>
+        <a:sysClr val="window" lastClr="FFFFFF"/>
+      </a:lt1>
+      <a:dk2>
+        <a:srgbClr val="1F497D"/>
+      </a:dk2>
+      <a:lt2>
+        <a:srgbClr val="EEECE1"/>
+      </a:lt2>
+      <a:accent1>
+        <a:srgbClr val="4F81BD"/>
+      </a:accent1>
+      <a:accent2>
+        <a:srgbClr val="C0504D"/>
+      </a:accent2>
+      <a:accent3>
+        <a:srgbClr val="9BBB59"/>
+      </a:accent3>
+      <a:accent4>
+        <a:srgbClr val="8064A2"/>
+      </a:accent4>
+      <a:accent5>
+        <a:srgbClr val="4BACC6"/>
+      </a:accent5>
+      <a:accent6>
+        <a:srgbClr val="F79646"/>
+      </a:accent6>
+      <a:hlink>
+        <a:srgbClr val="0000FF"/>
+      </a:hlink>
+      <a:folHlink>
+        <a:srgbClr val="800080"/>
+      </a:folHlink>
+    </a:clrScheme>
+    <a:fontScheme name="Office">
+      <a:majorFont>
+        <a:latin typeface="Cambria"/>
+        <a:ea typeface=""/>
+        <a:cs typeface=""/>
+        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
+        <a:font script="Hang" typeface="맑은 고딕"/>
+        <a:font script="Hans" typeface="宋体"/>
+        <a:font script="Hant" typeface="新細明體"/>
+        <a:font script="Arab" typeface="Times New Roman"/>
+        <a:font script="Hebr" typeface="Times New Roman"/>
+        <a:font script="Thai" typeface="Tahoma"/>
+        <a:font script="Ethi" typeface="Nyala"/>
+        <a:font script="Beng" typeface="Vrinda"/>
+        <a:font script="Gujr" typeface="Shruti"/>
+        <a:font script="Khmr" typeface="MoolBoran"/>
+        <a:font script="Knda" typeface="Tunga"/>
+        <a:font script="Guru" typeface="Raavi"/>
+        <a:font script="Cans" typeface="Euphemia"/>
+        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
+        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
+        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
+        <a:font script="Thaa" typeface="MV Boli"/>
+        <a:font script="Deva" typeface="Mangal"/>
+        <a:font script="Telu" typeface="Gautami"/>
+        <a:font script="Taml" typeface="Latha"/>
+        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
+        <a:font script="Orya" typeface="Kalinga"/>
+        <a:font script="Mlym" typeface="Kartika"/>
+        <a:font script="Laoo" typeface="DokChampa"/>
+        <a:font script="Sinh" typeface="Iskoola Pota"/>
+        <a:font script="Mong" typeface="Mongolian Baiti"/>
+        <a:font script="Viet" typeface="Times New Roman"/>
+        <a:font script="Uigh" typeface="Microsoft Uighur"/>
+      </a:majorFont>
+      <a:minorFont>
+        <a:latin typeface="Calibri"/>
+        <a:ea typeface=""/>
+        <a:cs typeface=""/>
+        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
+        <a:font script="Hang" typeface="맑은 고딕"/>
+        <a:font script="Hans" typeface="宋体"/>
+        <a:font script="Hant" typeface="新細明體"/>
+        <a:font script="Arab" typeface="Arial"/>
+        <a:font script="Hebr" typeface="Arial"/>
+        <a:font script="Thai" typeface="Tahoma"/>
+        <a:font script="Ethi" typeface="Nyala"/>
+        <a:font script="Beng" typeface="Vrinda"/>
+        <a:font script="Gujr" typeface="Shruti"/>
+        <a:font script="Khmr" typeface="DaunPenh"/>
+        <a:font script="Knda" typeface="Tunga"/>
+        <a:font script="Guru" typeface="Raavi"/>
+        <a:font script="Cans" typeface="Euphemia"/>
+        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
+        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
+        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
+        <a:font script="Thaa" typeface="MV Boli"/>
+        <a:font script="Deva" typeface="Mangal"/>
+        <a:font script="Telu" typeface="Gautami"/>
+        <a:font script="Taml" typeface="Latha"/>
+        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
+        <a:font script="Orya" typeface="Kalinga"/>
+        <a:font script="Mlym" typeface="Kartika"/>
+        <a:font script="Laoo" typeface="DokChampa"/>
+        <a:font script="Sinh" typeface="Iskoola Pota"/>
+        <a:font script="Mong" typeface="Mongolian Baiti"/>
+        <a:font script="Viet" typeface="Arial"/>
+        <a:font script="Uigh" typeface="Microsoft Uighur"/>
+      </a:minorFont>
+    </a:fontScheme>
+    <a:fmtScheme name="Office">
+      <a:fillStyleLst>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:gradFill rotWithShape="1">
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:tint val="50000"/>
+                <a:satMod val="300000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="35000">
+              <a:schemeClr val="phClr">
+                <a:tint val="37000"/>
+                <a:satMod val="300000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:tint val="15000"/>
+                <a:satMod val="350000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:lin ang="16200000" scaled="1"/>
+        </a:gradFill>
+        <a:gradFill rotWithShape="1">
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:shade val="51000"/>
+                <a:satMod val="130000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="80000">
+              <a:schemeClr val="phClr">
+                <a:shade val="93000"/>
+                <a:satMod val="130000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:shade val="94000"/>
+                <a:satMod val="135000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:lin ang="16200000" scaled="0"/>
+        </a:gradFill>
+      </a:fillStyleLst>
+      <a:lnStyleLst>
+        <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr">
+              <a:shade val="95000"/>
+              <a:satMod val="105000"/>
+            </a:schemeClr>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+        </a:ln>
+        <a:ln w="25400" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr"/>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+        </a:ln>
+        <a:ln w="38100" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr"/>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </a:lnStyleLst>
+      <a:effectStyleLst>
+        <a:effectStyle>
+          <a:effectLst>
+            <a:outerShdw blurRad="40000" dist="20000" dir="5400000" rotWithShape="0">
+              <a:srgbClr val="000000">
+                <a:alpha val="38000"/>
+              </a:srgbClr>
+            </a:outerShdw>
+          </a:effectLst>
+        </a:effectStyle>
+        <a:effectStyle>
+          <a:effectLst>
+            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
+              <a:srgbClr val="000000">
+                <a:alpha val="35000"/>
+              </a:srgbClr>
+            </a:outerShdw>
+          </a:effectLst>
+        </a:effectStyle>
+        <a:effectStyle>
+          <a:effectLst>
+            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
+              <a:srgbClr val="000000">
+                <a:alpha val="35000"/>
+              </a:srgbClr>
+            </a:outerShdw>
+          </a:effectLst>
+          <a:scene3d>
+            <a:camera prst="orthographicFront">
+              <a:rot lat="0" lon="0" rev="0"/>
+            </a:camera>
+            <a:lightRig rig="threePt" dir="t">
+              <a:rot lat="0" lon="0" rev="1200000"/>
+            </a:lightRig>
+          </a:scene3d>
+          <a:sp3d>
+            <a:bevelT w="63500" h="25400"/>
+          </a:sp3d>
+        </a:effectStyle>
+      </a:effectStyleLst>
+      <a:bgFillStyleLst>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:gradFill rotWithShape="1">
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:tint val="40000"/>
+                <a:satMod val="350000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="40000">
+              <a:schemeClr val="phClr">
+                <a:tint val="45000"/>
+                <a:shade val="99000"/>
+                <a:satMod val="350000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:shade val="20000"/>
+                <a:satMod val="255000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:path path="circle">
+            <a:fillToRect l="50000" t="-80000" r="50000" b="180000"/>
+          </a:path>
+        </a:gradFill>
+        <a:gradFill rotWithShape="1">
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:tint val="80000"/>
+                <a:satMod val="300000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:shade val="30000"/>
+                <a:satMod val="200000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:path path="circle">
+            <a:fillToRect l="50000" t="50000" r="50000" b="50000"/>
+          </a:path>
+        </a:gradFill>
+      </a:bgFillStyleLst>
+    </a:fmtScheme>
+  </a:themeElements>
+  <a:objectDefaults/>
+  <a:extraClrSchemeLst/>
+</a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:I53"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="60" customWidth="1" min="3" max="3"/>
+    <col width="80" customWidth="1" min="5" max="5"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
@@ -65,12 +470,12 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2024-01-08</t>
+          <t>2026-01-05</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Meeting #1</t>
+          <t>2026-01-05 — Volta-7 Ramp Kickoff and Milestone Alignment</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -95,12 +500,12 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>2024-01-10</t>
+          <t>2026-01-07</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>2024-01-10</t>
+          <t>2026-01-07</t>
         </is>
       </c>
     </row>
@@ -112,12 +517,12 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2024-01-08</t>
+          <t>2026-01-05</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Meeting #1</t>
+          <t>2026-01-05 — Volta-7 Ramp Kickoff and Milestone Alignment</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -142,12 +547,12 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>2024-01-11</t>
+          <t>2026-01-08</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>2024-01-11</t>
+          <t>2026-01-08</t>
         </is>
       </c>
     </row>
@@ -159,12 +564,12 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2024-01-15</t>
+          <t>2026-01-12</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Meeting #2</t>
+          <t>2026-01-12 — First Silicon Yield Review — Lot LOT-V7-001</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -189,12 +594,12 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>2024-01-17</t>
+          <t>2026-01-14</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>2024-01-16</t>
+          <t>2026-01-13</t>
         </is>
       </c>
     </row>
@@ -206,12 +611,12 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>2024-01-15</t>
+          <t>2026-01-12</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Meeting #2</t>
+          <t>2026-01-12 — First Silicon Yield Review — Lot LOT-V7-001</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -236,12 +641,12 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>2024-01-22</t>
+          <t>2026-01-19</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>2024-01-21</t>
+          <t>2026-01-18</t>
         </is>
       </c>
     </row>
@@ -253,12 +658,12 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>2024-01-22</t>
+          <t>2026-01-19</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Meeting #3</t>
+          <t>2026-01-19 — ATE Test Program Readiness and Vector Validation</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -283,12 +688,12 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>2024-01-26</t>
+          <t>2026-01-23</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>2024-01-26</t>
+          <t>2026-01-23</t>
         </is>
       </c>
     </row>
@@ -300,12 +705,12 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>2024-01-22</t>
+          <t>2026-01-19</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Meeting #3</t>
+          <t>2026-01-19 — ATE Test Program Readiness and Vector Validation</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -330,12 +735,12 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>2024-01-23</t>
+          <t>2026-01-20</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>2024-01-23</t>
+          <t>2026-01-20</t>
         </is>
       </c>
     </row>
@@ -347,12 +752,12 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>2024-01-29</t>
+          <t>2026-01-26</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Meeting #4</t>
+          <t>2026-01-26 — Design-to-Product Engineering Handoff Alignment</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -377,12 +782,12 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>2024-02-02</t>
+          <t>2026-01-30</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>2024-02-02</t>
+          <t>2026-01-30</t>
         </is>
       </c>
     </row>
@@ -394,12 +799,12 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>2024-01-29</t>
+          <t>2026-01-26</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Meeting #4</t>
+          <t>2026-01-26 — Design-to-Product Engineering Handoff Alignment</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -424,12 +829,12 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>2024-02-05</t>
+          <t>2026-02-02</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>2024-02-04</t>
+          <t>2026-02-01</t>
         </is>
       </c>
     </row>
@@ -441,12 +846,12 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>2024-02-05</t>
+          <t>2026-02-02</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Meeting #5</t>
+          <t>2026-02-02 — Yield Review &amp; Failure Analysis Readout — Metal 3 CMP Defect</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -456,7 +861,7 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Track split-lot split run on Lot LOT-V7-006 with modified CMP recipe in yield tracker</t>
+          <t>Track the first full-recipe run on Lot LOT-V7-006 (2.1 psi + Slurry B-4) in the yield tracker</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
@@ -471,12 +876,12 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>2024-02-09</t>
+          <t>2026-02-06</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>2024-02-09</t>
+          <t>2026-02-06</t>
         </is>
       </c>
     </row>
@@ -488,12 +893,12 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>2024-02-05</t>
+          <t>2026-02-02</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Meeting #5</t>
+          <t>2026-02-02 — Yield Review &amp; Failure Analysis Readout — Metal 3 CMP Defect</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -518,12 +923,12 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>2024-02-12</t>
+          <t>2026-02-09</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>2024-02-11</t>
+          <t>2026-02-08</t>
         </is>
       </c>
     </row>
@@ -535,27 +940,27 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>2024-02-12</t>
+          <t>2026-02-04</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Meeting #6</t>
+          <t>2026-02-04 — CMP Slurry Supply &amp; Second-Source Qualification — Slurry B-4</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Kevin Tran</t>
+          <t>Nadia Rahman</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Load 231 units into HTOL stress chambers and verify bias supply voltages</t>
+          <t>Place the expedite order with Kestrel Materials and set a 30-day minimum safety stock for Slurry B-4</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>Critical</t>
+          <t>High</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
@@ -565,12 +970,12 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>2024-02-16</t>
+          <t>2026-02-06</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>2024-02-16</t>
+          <t>2026-02-06</t>
         </is>
       </c>
     </row>
@@ -582,27 +987,27 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>2024-02-12</t>
+          <t>2026-02-04</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Meeting #6</t>
+          <t>2026-02-04 — CMP Slurry Supply &amp; Second-Source Qualification — Slurry B-4</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Anna Becker</t>
+          <t>Wei Lim</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Review and archive chamber calibration certificates and qual travelers in QMS</t>
+          <t>Run three Halvorsen slurry split lots with post-M3 inline inspection</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
@@ -612,12 +1017,12 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>2024-02-18</t>
+          <t>2026-03-27</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>2024-02-17</t>
+          <t>2026-03-26</t>
         </is>
       </c>
     </row>
@@ -629,27 +1034,27 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>2024-02-19</t>
+          <t>2026-02-04</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Meeting #7</t>
+          <t>2026-02-04 — CMP Slurry Supply &amp; Second-Source Qualification — Slurry B-4</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Emma White</t>
+          <t>James Ortiz</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Execute ATE screening on 80 packaged units to select 50 golden samples</t>
+          <t>Correlate Halvorsen split-lot sort yield against Slurry B-4 in the yield tracker</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>Critical</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
@@ -659,12 +1064,12 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>2024-02-27</t>
+          <t>2026-04-03</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>2024-02-26</t>
+          <t>2026-04-02</t>
         </is>
       </c>
     </row>
@@ -676,22 +1081,22 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>2024-02-19</t>
+          <t>2026-02-09</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Meeting #7</t>
+          <t>2026-02-09 — Volta-7 Automotive Reliability Qualification Plan Review</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Tom Harris</t>
+          <t>Kevin Tran</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Draft customer sample release memo with operating waivers and deliver to NovaDrive</t>
+          <t>Load 231 units into HTOL stress chambers and verify bias supply voltages</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
@@ -706,12 +1111,12 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>2024-02-28</t>
+          <t>2026-02-13</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>2024-02-28</t>
+          <t>2026-02-13</t>
         </is>
       </c>
     </row>
@@ -723,27 +1128,27 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>2024-02-26</t>
+          <t>2026-02-09</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Meeting #8</t>
+          <t>2026-02-09 — Volta-7 Automotive Reliability Qualification Plan Review</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Emma White</t>
+          <t>Anna Becker</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Parallelize dual ADC linearity routines to shave 350ms off ATE test time</t>
+          <t>Review and archive chamber calibration certificates and qual travelers in QMS</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
@@ -753,12 +1158,12 @@
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>2024-03-05</t>
+          <t>2026-02-15</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>2024-03-04</t>
+          <t>2026-02-14</t>
         </is>
       </c>
     </row>
@@ -770,22 +1175,22 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>2024-02-26</t>
+          <t>2026-02-16</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Meeting #8</t>
+          <t>2026-02-16 — Customer Escalation — NovaDrive Engineering Sample Demand</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Derek Cole</t>
+          <t>Emma White</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Coordinate dispatch of 50 ES1 units via express courier to NovaDrive Motors</t>
+          <t>Execute ATE screening on 80 packaged units to select 50 golden samples</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
@@ -800,12 +1205,12 @@
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>2024-02-28</t>
+          <t>2026-02-24</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>2024-02-28</t>
+          <t>2026-02-23</t>
         </is>
       </c>
     </row>
@@ -817,22 +1222,22 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>2024-03-04</t>
+          <t>2026-02-16</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Meeting #9</t>
+          <t>2026-02-16 — Customer Escalation — NovaDrive Engineering Sample Demand</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Kevin Tran</t>
+          <t>Tom Harris</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Complete 500-hour HTOL pull and execute tri-temp ATE electrical screening</t>
+          <t>Draft customer sample release memo with operating waivers and deliver to NovaDrive</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
@@ -847,12 +1252,12 @@
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>2024-03-11</t>
+          <t>2026-02-25</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>2024-03-11</t>
+          <t>2026-02-25</t>
         </is>
       </c>
     </row>
@@ -864,27 +1269,27 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>2024-03-04</t>
+          <t>2026-02-23</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Meeting #9</t>
+          <t>2026-02-23 — ATE Test Program Release and Execution Time Review</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Derek Cole</t>
+          <t>Emma White</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Prepare customer PPAP documentation schedule assuming successful 500h gate</t>
+          <t>Parallelize dual ADC linearity routines to shave 350ms off ATE test time</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
@@ -894,12 +1299,12 @@
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>2024-03-08</t>
+          <t>2026-03-03</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>2024-03-08</t>
+          <t>2026-03-02</t>
         </is>
       </c>
     </row>
@@ -911,22 +1316,22 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>2024-03-11</t>
+          <t>2026-02-23</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Meeting #10</t>
+          <t>2026-02-23 — ATE Test Program Release and Execution Time Review</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Rosa Santos</t>
+          <t>Derek Cole</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Perform decapsulation, EMMI hotspot detection, and FIB cross-section on failing units</t>
+          <t>Coordinate dispatch of 50 ES1 units via express courier to NovaDrive Motors</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
@@ -941,12 +1346,12 @@
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>2024-03-13</t>
+          <t>2026-02-25</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>2024-03-13</t>
+          <t>2026-02-25</t>
         </is>
       </c>
     </row>
@@ -958,12 +1363,12 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>2024-03-11</t>
+          <t>2026-03-02</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Meeting #10</t>
+          <t>2026-03-02 — Volta-7 Program Status Check &amp; Risk Review</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
@@ -973,7 +1378,7 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>Quarantine remaining 228 HTOL units and preserve chamber bias and environmental logs</t>
+          <t>Complete 500-hour HTOL pull and execute tri-temp ATE electrical screening</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
@@ -988,12 +1393,12 @@
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>2024-03-12</t>
+          <t>2026-03-09</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>2024-03-12</t>
+          <t>2026-03-09</t>
         </is>
       </c>
     </row>
@@ -1005,27 +1410,27 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>2024-03-14</t>
+          <t>2026-03-02</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Meeting #11</t>
+          <t>2026-03-02 — Volta-7 Program Status Check &amp; Risk Review</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Rosa Santos</t>
+          <t>Derek Cole</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>Finalize and distribute formal Failure Analysis Report FA-2024-0314</t>
+          <t>Prepare customer PPAP documentation schedule assuming successful 500h gate</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>Critical</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
@@ -1035,12 +1440,12 @@
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>2024-03-15</t>
+          <t>2026-03-06</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>2024-03-14</t>
+          <t>2026-03-06</t>
         </is>
       </c>
     </row>
@@ -1052,22 +1457,22 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>2024-03-14</t>
+          <t>2026-03-09</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Meeting #11</t>
+          <t>2026-03-09 — CRITICAL ALERT: HTOL 500-Hour Intermediate Readout Failure</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Sara Nolan</t>
+          <t>Rosa Santos</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>Pull design schematic and layout database for IO clamp replacement with automotive-grade 280µm cell</t>
+          <t>Perform decapsulation, EMMI hotspot detection, and FIB cross-section on failing units</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
@@ -1082,12 +1487,12 @@
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>2024-03-16</t>
+          <t>2026-03-11</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>2024-03-15</t>
+          <t>2026-03-11</t>
         </is>
       </c>
     </row>
@@ -1099,22 +1504,22 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>2024-03-18</t>
+          <t>2026-03-09</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Meeting #12</t>
+          <t>2026-03-09 — CRITICAL ALERT: HTOL 500-Hour Intermediate Readout Failure</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Anna Becker</t>
+          <t>Kevin Tran</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>Lead 8D Corrective Action Report generation and coordinate technical exhibits with Rosa Santos</t>
+          <t>Quarantine remaining 228 HTOL units and preserve chamber bias and environmental logs</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
@@ -1129,12 +1534,12 @@
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>2024-04-05</t>
+          <t>2026-03-10</t>
         </is>
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>2024-04-05</t>
+          <t>2026-03-10</t>
         </is>
       </c>
     </row>
@@ -1146,22 +1551,22 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>2024-03-18</t>
+          <t>2026-03-12</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Meeting #12</t>
+          <t>2026-03-12 — Emergency Failure Analysis Readout — HTOL Root Cause</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Tom Harris</t>
+          <t>Rosa Santos</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>Issue formal executive response letter to Marcus Vance at NovaDrive Motors</t>
+          <t>Finalize and distribute formal Failure Analysis Report FA-2026-0312</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
@@ -1176,12 +1581,12 @@
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>2024-03-20</t>
+          <t>2026-03-13</t>
         </is>
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>2024-03-19</t>
+          <t>2026-03-12</t>
         </is>
       </c>
     </row>
@@ -1193,12 +1598,12 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>2024-03-22</t>
+          <t>2026-03-12</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Meeting #13</t>
+          <t>2026-03-12 — Emergency Failure Analysis Readout — HTOL Root Cause</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
@@ -1208,7 +1613,7 @@
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>Complete DRC/LVS physical verification and release Rev B mask stream tape-out</t>
+          <t>Pull design schematic and layout database for IO clamp replacement with automotive-grade 280µm cell</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
@@ -1223,12 +1628,12 @@
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>2024-03-23</t>
+          <t>2026-03-14</t>
         </is>
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>2024-03-23</t>
+          <t>2026-03-13</t>
         </is>
       </c>
     </row>
@@ -1240,22 +1645,22 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>2024-03-22</t>
+          <t>2026-03-16</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Meeting #13</t>
+          <t>2026-03-16 — NovaDrive Executive Escalation — HTOL Failure Notification</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>James Ortiz</t>
+          <t>Anna Becker</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>Coordinate hot-lot expedition protocol with Penang fab operations</t>
+          <t>Lead 8D Corrective Action Report generation and coordinate technical exhibits with Rosa Santos</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
@@ -1270,12 +1675,12 @@
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>2024-03-25</t>
+          <t>2026-04-03</t>
         </is>
       </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>2024-03-24</t>
+          <t>2026-04-03</t>
         </is>
       </c>
     </row>
@@ -1287,27 +1692,27 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>2024-03-29</t>
+          <t>2026-03-16</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Meeting #14</t>
+          <t>2026-03-16 — NovaDrive Executive Escalation — HTOL Failure Notification</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Derek Cole</t>
+          <t>Tom Harris</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>Monitor daily Penang fab WIP velocity for Lot LOT-V7-020 and provide morning updates</t>
+          <t>Issue formal executive response letter to Marcus Vance at NovaDrive Motors</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Critical</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
@@ -1317,12 +1722,12 @@
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>2024-04-03</t>
+          <t>2026-03-18</t>
         </is>
       </c>
       <c r="I28" t="inlineStr">
         <is>
-          <t>2024-04-03</t>
+          <t>2026-03-17</t>
         </is>
       </c>
     </row>
@@ -1334,27 +1739,27 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>2024-03-29</t>
+          <t>2026-03-20</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Meeting #14</t>
+          <t>2026-03-20 — Volta-7 Rev B Silicon Mask Fix &amp; Execution Strategy</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Anna Becker</t>
+          <t>Sara Nolan</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>Finalize 8D report draft with Rosa's FA imagery for executive review</t>
+          <t>Complete DRC/LVS physical verification and release Rev B mask stream tape-out</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Critical</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
@@ -1364,12 +1769,12 @@
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>2024-04-05</t>
+          <t>2026-03-21</t>
         </is>
       </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>2024-04-05</t>
+          <t>2026-03-21</t>
         </is>
       </c>
     </row>
@@ -1381,22 +1786,22 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>2024-04-07</t>
+          <t>2026-03-20</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Meeting #15</t>
+          <t>2026-03-20 — Volta-7 Rev B Silicon Mask Fix &amp; Execution Strategy</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Tom Harris</t>
+          <t>James Ortiz</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>Transmit signed 8D report to NovaDrive executive quality management</t>
+          <t>Coordinate hot-lot expedition protocol with Penang fab operations</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
@@ -1411,12 +1816,12 @@
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>2024-04-08</t>
+          <t>2026-03-23</t>
         </is>
       </c>
       <c r="I30" t="inlineStr">
         <is>
-          <t>2024-04-07</t>
+          <t>2026-03-22</t>
         </is>
       </c>
     </row>
@@ -1428,27 +1833,27 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>2024-04-07</t>
+          <t>2026-03-27</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Meeting #15</t>
+          <t>2026-03-27 — Rev B Silicon Timeline &amp; Critical Path Risk Assessment</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Anna Becker</t>
+          <t>Derek Cole</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>Log 8D submission into FastChip customer CAR tracking database</t>
+          <t>Monitor daily Penang fab WIP velocity for Lot LOT-V7-020 and provide morning updates</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
@@ -1458,12 +1863,12 @@
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>2024-04-08</t>
+          <t>2026-04-01</t>
         </is>
       </c>
       <c r="I31" t="inlineStr">
         <is>
-          <t>2024-04-08</t>
+          <t>2026-04-01</t>
         </is>
       </c>
     </row>
@@ -1475,22 +1880,22 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>2024-04-21</t>
+          <t>2026-03-27</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Meeting #16</t>
+          <t>2026-03-27 — Rev B Silicon Timeline &amp; Critical Path Risk Assessment</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>James Ortiz</t>
+          <t>Anna Becker</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>Update yield tracker with complete 25-wafer sort results for Lot LOT-V7-020</t>
+          <t>Finalize 8D report draft with Rosa's FA imagery for executive review</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
@@ -1505,12 +1910,12 @@
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>2024-04-23</t>
+          <t>2026-04-03</t>
         </is>
       </c>
       <c r="I32" t="inlineStr">
         <is>
-          <t>2024-04-22</t>
+          <t>2026-04-03</t>
         </is>
       </c>
     </row>
@@ -1522,22 +1927,22 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>2024-04-21</t>
+          <t>2026-04-05</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Meeting #16</t>
+          <t>2026-04-05 — Final Review of 8D Corrective Action Report for NovaDrive</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>Emma White</t>
+          <t>Tom Harris</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>Hand off 500 tested dies to fast-track packaging for reliability qual build</t>
+          <t>Transmit signed 8D report to NovaDrive executive quality management</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
@@ -1552,12 +1957,12 @@
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>2024-04-22</t>
+          <t>2026-04-06</t>
         </is>
       </c>
       <c r="I33" t="inlineStr">
         <is>
-          <t>2024-04-22</t>
+          <t>2026-04-05</t>
         </is>
       </c>
     </row>
@@ -1569,27 +1974,27 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>2024-04-28</t>
+          <t>2026-04-05</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Meeting #17</t>
+          <t>2026-04-05 — Final Review of 8D Corrective Action Report for NovaDrive</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>Kevin Tran</t>
+          <t>Anna Becker</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>Publish completed Reliability Qualification Summary Report and sign off certificate</t>
+          <t>Log 8D submission into FastChip customer CAR tracking database</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>Critical</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
@@ -1599,12 +2004,12 @@
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>2024-04-30</t>
+          <t>2026-04-06</t>
         </is>
       </c>
       <c r="I34" t="inlineStr">
         <is>
-          <t>2024-04-30</t>
+          <t>2026-04-06</t>
         </is>
       </c>
     </row>
@@ -1616,27 +2021,27 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>2024-04-28</t>
+          <t>2026-04-19</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Meeting #17</t>
+          <t>2026-04-19 — Rev B Silicon First Wafer Sort Yield Readout</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>Anna Becker</t>
+          <t>James Ortiz</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>Update 8D report with D6 closure data and submit validation package to NovaDrive</t>
+          <t>Update yield tracker with complete 25-wafer sort results for Lot LOT-V7-020</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>Critical</t>
+          <t>High</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
@@ -1646,12 +2051,12 @@
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>2024-04-30</t>
+          <t>2026-04-21</t>
         </is>
       </c>
       <c r="I35" t="inlineStr">
         <is>
-          <t>2024-04-30</t>
+          <t>2026-04-20</t>
         </is>
       </c>
     </row>
@@ -1663,27 +2068,27 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>2024-05-05</t>
+          <t>2026-04-19</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Meeting #18</t>
+          <t>2026-04-19 — Rev B Silicon First Wafer Sort Yield Readout</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>Anna Becker</t>
+          <t>Emma White</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>Conduct internal dry-run audit with all track owners and verify traveler archives</t>
+          <t>Hand off 500 tested dies to fast-track packaging for reliability qual build</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Critical</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
@@ -1693,12 +2098,12 @@
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>2024-05-08</t>
+          <t>2026-04-20</t>
         </is>
       </c>
       <c r="I36" t="inlineStr">
         <is>
-          <t>2024-05-08</t>
+          <t>2026-04-20</t>
         </is>
       </c>
     </row>
@@ -1710,27 +2115,27 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>2024-05-05</t>
+          <t>2026-04-26</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Meeting #18</t>
+          <t>2026-04-26 — Rev B Early Reliability Readout — ELFR &amp; HAST</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>Tom Harris</t>
+          <t>Kevin Tran</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>Finalize audit agenda and logistics with NovaDrive audit delegation</t>
+          <t>Run the 168h and 500h HTOL pulls and publish the Reliability Qualification Summary after the 1000-hour readout</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Critical</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
@@ -1740,12 +2145,12 @@
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>2024-05-09</t>
+          <t>2026-06-03</t>
         </is>
       </c>
       <c r="I37" t="inlineStr">
         <is>
-          <t>2024-05-09</t>
+          <t>2026-06-03</t>
         </is>
       </c>
     </row>
@@ -1757,12 +2162,12 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>2024-05-13</t>
+          <t>2026-04-26</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Meeting #19</t>
+          <t>2026-04-26 — Rev B Early Reliability Readout — ELFR &amp; HAST</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
@@ -1772,12 +2177,12 @@
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>Submit formal corrective action response for the two minor audit observations to NovaDrive</t>
+          <t>Send interim D6 validation package (ELFR, HAST) to NovaDrive</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Critical</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
@@ -1787,12 +2192,12 @@
       </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t>2024-05-20</t>
+          <t>2026-04-28</t>
         </is>
       </c>
       <c r="I38" t="inlineStr">
         <is>
-          <t>2024-05-18</t>
+          <t>2026-04-28</t>
         </is>
       </c>
     </row>
@@ -1804,27 +2209,27 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>2024-05-13</t>
+          <t>2026-05-03</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Meeting #19</t>
+          <t>2026-05-03 — NovaDrive On-Site Quality Audit Readiness &amp; Role Assignment</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>Derek Cole</t>
+          <t>Anna Becker</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>Release production purchase order schedule to Penang fab for 200k unit monthly volume</t>
+          <t>Conduct internal dry-run audit with all track owners and verify traveler archives</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>Critical</t>
+          <t>High</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
@@ -1834,12 +2239,12 @@
       </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t>2024-05-16</t>
+          <t>2026-05-06</t>
         </is>
       </c>
       <c r="I39" t="inlineStr">
         <is>
-          <t>2024-05-15</t>
+          <t>2026-05-06</t>
         </is>
       </c>
     </row>
@@ -1851,22 +2256,22 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>2024-05-20</t>
+          <t>2026-05-03</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>Meeting #20</t>
+          <t>2026-05-03 — NovaDrive On-Site Quality Audit Readiness &amp; Role Assignment</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>Lisa Park</t>
+          <t>Tom Harris</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>Update PE Division SOP-PE-042 with enhanced design handoff and reliability qual protocols</t>
+          <t>Finalize audit agenda and logistics with NovaDrive audit delegation</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
@@ -1881,12 +2286,12 @@
       </c>
       <c r="H40" t="inlineStr">
         <is>
-          <t>2024-05-27</t>
+          <t>2026-05-07</t>
         </is>
       </c>
       <c r="I40" t="inlineStr">
         <is>
-          <t>2024-05-25</t>
+          <t>2026-05-07</t>
         </is>
       </c>
     </row>
@@ -1898,45 +2303,595 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>2024-05-20</t>
+          <t>2026-05-11</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Meeting #20</t>
+          <t>2026-05-11 — PE Division All-Hands — NovaDrive Audit Outcome &amp; Production Release</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
+          <t>Anna Becker</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>Submit formal corrective action response for the two minor audit observations to NovaDrive</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>2026-05-18</t>
+        </is>
+      </c>
+      <c r="I41" t="inlineStr">
+        <is>
+          <t>2026-05-16</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>ACT-041</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>2026-05-11</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>2026-05-11 — PE Division All-Hands — NovaDrive Audit Outcome &amp; Production Release</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>Derek Cole</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>Release production purchase order schedule to Penang fab for 200k unit monthly volume</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="I42" t="inlineStr">
+        <is>
+          <t>2026-05-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>ACT-042</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>2026-05-18</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>2026-05-18 — Volta-7 Program Retrospective &amp; Lessons Learned</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>Lisa Park</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>Update PE Division SOP-PE-042 with enhanced design handoff and reliability qual protocols</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="H43" t="inlineStr">
+        <is>
+          <t>2026-05-25</t>
+        </is>
+      </c>
+      <c r="I43" t="inlineStr">
+        <is>
+          <t>2026-05-23</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>ACT-043</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>2026-05-18</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>2026-05-18 — Volta-7 Program Retrospective &amp; Lessons Learned</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
           <t>Sara Nolan</t>
         </is>
       </c>
-      <c r="E41" t="inlineStr">
+      <c r="E44" t="inlineStr">
         <is>
           <t>Implement automated automotive ESD DRC rule decks across CAD tool flows</t>
         </is>
       </c>
-      <c r="F41" t="inlineStr">
+      <c r="F44" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="G41" t="inlineStr">
-        <is>
-          <t>Closed</t>
-        </is>
-      </c>
-      <c r="H41" t="inlineStr">
-        <is>
-          <t>2024-05-30</t>
-        </is>
-      </c>
-      <c r="I41" t="inlineStr">
-        <is>
-          <t>2024-05-28</t>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="H44" t="inlineStr">
+        <is>
+          <t>2026-05-28</t>
+        </is>
+      </c>
+      <c r="I44" t="inlineStr">
+        <is>
+          <t>2026-05-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>ACT-044</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>2026-05-20</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>2026-05-20 — Volta-7 Production Ramp — Capacity &amp; Supply Readiness</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>Nadia Rahman</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>Issue the Meridian Packaging qualification purchase order and secure July leadframe allocation</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="H45" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="I45" t="inlineStr">
+        <is>
+          <t>2026-05-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>ACT-045</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>2026-05-20</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>2026-05-20 — Volta-7 Production Ramp — Capacity &amp; Supply Readiness</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>Kevin Tran</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>Run MSL3 preconditioning, TC and C-SAM on three Meridian leadframe assembly lots</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="G46" t="inlineStr">
+        <is>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="H46" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="I46" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>ACT-046</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>2026-05-20</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>2026-05-20 — Volta-7 Production Ramp — Capacity &amp; Supply Readiness</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>Wei Lim</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>Release Tester 04 to production and confirm the 250 wafer starts/month plan</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="G47" t="inlineStr">
+        <is>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="H47" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="I47" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>ACT-047</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>2026-06-02</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>2026-06-02 — Rev B 1000-Hour HTOL Final Readout &amp; Full Qualification</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>Kevin Tran</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>Publish the Reliability Qualification Summary and the final reliability test matrix</t>
+        </is>
+      </c>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="G48" t="inlineStr">
+        <is>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="H48" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
+      <c r="I48" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>ACT-048</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>2026-06-02</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>2026-06-02 — Rev B 1000-Hour HTOL Final Readout &amp; Full Qualification</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>Anna Becker</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>Submit the final D6 validation package and close CAR-2026-ND01 with NovaDrive</t>
+        </is>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="G49" t="inlineStr">
+        <is>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="H49" t="inlineStr">
+        <is>
+          <t>2026-06-04</t>
+        </is>
+      </c>
+      <c r="I49" t="inlineStr">
+        <is>
+          <t>2026-06-04</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>ACT-049</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>2026-06-02</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>2026-06-02 — Rev B 1000-Hour HTOL Final Readout &amp; Full Qualification</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>Tom Harris</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>Obtain the full PSW signature from Marcus Vance at NovaDrive</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="G50" t="inlineStr">
+        <is>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="H50" t="inlineStr">
+        <is>
+          <t>2026-06-05</t>
+        </is>
+      </c>
+      <c r="I50" t="inlineStr">
+        <is>
+          <t>2026-06-05</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>ACT-050</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>2026-09-15 — FY2027 Strategy Review — Volta-8 Roadmap &amp; Product Portfolio</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>Amanda Foster</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>Publish Volta-8 product requirements and a staffing plan with PE in the design reviews</t>
+        </is>
+      </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="G51" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="H51" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>ACT-051</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>2026-09-15 — FY2027 Strategy Review — Volta-8 Roadmap &amp; Product Portfolio</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>Kevin Nash</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>Release the FY2027 budget including Volta-8 funding and Penang capacity expansion</t>
+        </is>
+      </c>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="G52" t="inlineStr">
+        <is>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="H52" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>ACT-052</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>2026-09-15 — FY2027 Strategy Review — Volta-8 Roadmap &amp; Product Portfolio</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>Mike Chen</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>Report the status of the two Tier-1 Volta-7 evaluations with Tom Harris</t>
+        </is>
+      </c>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="G53" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="H53" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
         </is>
       </c>
     </row>
   </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>